<commit_message>
fix: repair workbook required header styles
</commit_message>
<xml_diff>
--- a/templates/izi-park-product-owner-workbook.xlsx
+++ b/templates/izi-park-product-owner-workbook.xlsx
@@ -418,6 +418,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7C2D12"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -468,6 +474,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>